<commit_message>
feat: update UI + CMS
</commit_message>
<xml_diff>
--- a/template/fractional-cc/List sản phẩm fractional CC.xlsx
+++ b/template/fractional-cc/List sản phẩm fractional CC.xlsx
@@ -604,7 +604,7 @@
     <xdr:ext cx="1981200" cy="2076450"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image6.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -632,7 +632,7 @@
     <xdr:ext cx="1952625" cy="1714500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image9.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -660,7 +660,7 @@
     <xdr:ext cx="1743075" cy="1933575"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image8.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image10.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -688,7 +688,7 @@
     <xdr:ext cx="1981200" cy="2162175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -744,7 +744,7 @@
     <xdr:ext cx="1714500" cy="1876425"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image9.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -772,7 +772,7 @@
     <xdr:ext cx="1914525" cy="2247900"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -800,7 +800,7 @@
     <xdr:ext cx="1790700" cy="2028825"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image7.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -828,7 +828,7 @@
     <xdr:ext cx="1866900" cy="2143125"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image10.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image8.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -856,7 +856,7 @@
     <xdr:ext cx="1971675" cy="2295525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image7.png" title="Hình ảnh"/>
+        <xdr:cNvPr id="0" name="image5.png" title="Hình ảnh"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>

</xml_diff>